<commit_message>
Pub list update and Bonaire/Curacao added
</commit_message>
<xml_diff>
--- a/pubs/2026 Pubs.xlsx
+++ b/pubs/2026 Pubs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\WebSite\pubs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2846DBDD-90E4-4EB5-A0F4-AFC5F86A3096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{993E71EA-5340-4E8B-BF1D-7F364AF596B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA8581EE-2B0A-489C-80E8-4550A4BD8B73}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="21132" windowHeight="8880" activeTab="1" xr2:uid="{AA8581EE-2B0A-489C-80E8-4550A4BD8B73}"/>
   </bookViews>
   <sheets>
     <sheet name="UK" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="227">
   <si>
     <t>London</t>
   </si>
@@ -704,6 +704,18 @@
   </si>
   <si>
     <t>Woolhampton</t>
+  </si>
+  <si>
+    <t>The Mill House</t>
+  </si>
+  <si>
+    <t>North Warnborough</t>
+  </si>
+  <si>
+    <t>cw</t>
+  </si>
+  <si>
+    <t>bq</t>
   </si>
 </sst>
 </file>
@@ -1235,7 +1247,7 @@
       </c>
       <c r="G3" s="10">
         <f>COUNTIF(C:C, "&lt;&gt;") - 1</f>
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -1283,7 +1295,7 @@
       </c>
       <c r="G5" s="12">
         <f>G3+G4</f>
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3097,6 +3109,15 @@
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" s="8">
         <v>113</v>
+      </c>
+      <c r="B114" s="1">
+        <v>46168</v>
+      </c>
+      <c r="C114" t="s">
+        <v>223</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
@@ -4895,10 +4916,16 @@
       <c r="A63" s="8">
         <v>62</v>
       </c>
+      <c r="E63" s="2" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="8">
         <v>63</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Update to pub list
</commit_message>
<xml_diff>
--- a/pubs/2026 Pubs.xlsx
+++ b/pubs/2026 Pubs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\WebSite\pubs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47B8ECA-0FC3-4257-A3E2-D4D0942F56E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0858A61-E7EF-4DD6-B1EF-0B09CC84A9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA8581EE-2B0A-489C-80E8-4550A4BD8B73}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="260">
   <si>
     <t>London</t>
   </si>
@@ -806,6 +806,15 @@
   </si>
   <si>
     <t>gb</t>
+  </si>
+  <si>
+    <t>Sherborne St John</t>
+  </si>
+  <si>
+    <t>The Crown</t>
+  </si>
+  <si>
+    <t>The George &amp; Horn</t>
   </si>
 </sst>
 </file>
@@ -1349,7 +1358,7 @@
       </c>
       <c r="G3" s="10">
         <f>COUNTIF(C:C, "&lt;&gt;") - 1</f>
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -1397,7 +1406,7 @@
       </c>
       <c r="G5" s="12">
         <f>G3+G4</f>
-        <v>195</v>
+        <v>198</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3502,15 +3511,51 @@
       <c r="A119" s="8">
         <v>118</v>
       </c>
+      <c r="B119" s="1">
+        <v>46214</v>
+      </c>
+      <c r="C119" t="s">
+        <v>227</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E119" s="17" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" s="8">
         <v>119</v>
       </c>
+      <c r="B120" s="1">
+        <v>46214</v>
+      </c>
+      <c r="C120" t="s">
+        <v>258</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E120" s="17" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" s="8">
         <v>120</v>
+      </c>
+      <c r="B121" s="1">
+        <v>46214</v>
+      </c>
+      <c r="C121" t="s">
+        <v>259</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E121" s="17" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Commas added to large numbers in annual stats
</commit_message>
<xml_diff>
--- a/pubs/2026 Pubs.xlsx
+++ b/pubs/2026 Pubs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\WebSite\pubs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16AD6FE6-2F36-4276-B549-9761890FAEDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E19B36-4C92-472C-AF1E-D951065632D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA8581EE-2B0A-489C-80E8-4550A4BD8B73}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="266">
   <si>
     <t>London</t>
   </si>
@@ -827,6 +827,12 @@
   </si>
   <si>
     <t>Whitway</t>
+  </si>
+  <si>
+    <t>The Bricklayers Arms</t>
+  </si>
+  <si>
+    <t>Parched</t>
   </si>
 </sst>
 </file>
@@ -1370,7 +1376,7 @@
       </c>
       <c r="G3" s="10">
         <f>COUNTIF(C:C, "&lt;&gt;") - 1</f>
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -1418,7 +1424,7 @@
       </c>
       <c r="G5" s="12">
         <f>G3+G4</f>
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -3608,10 +3614,34 @@
       <c r="A124" s="8">
         <v>123</v>
       </c>
+      <c r="B124" s="1">
+        <v>46220</v>
+      </c>
+      <c r="C124" t="s">
+        <v>264</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E124" s="17" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" s="8">
         <v>124</v>
+      </c>
+      <c r="B125" s="1">
+        <v>46220</v>
+      </c>
+      <c r="C125" t="s">
+        <v>265</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E125" s="17" t="s">
+        <v>256</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>